<commit_message>
implementada tabla competidores y facebook
</commit_message>
<xml_diff>
--- a/projecto_centralizar/frontend/public/templates/contacts_import_template.xlsx
+++ b/projecto_centralizar/frontend/public/templates/contacts_import_template.xlsx
@@ -22,28 +22,28 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
-    <t xml:space="preserve">empresa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nombre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">apellido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">linkedin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">telefono</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">campaña</t>
+    <t xml:space="preserve">Nombre empresa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apellidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LinkedIn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telefono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaña</t>
   </si>
   <si>
     <t xml:space="preserve">Acme SL</t>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">Head of Sales</t>
   </si>
   <si>
-    <t xml:space="preserve">Campaña20</t>
+    <t xml:space="preserve">Campaña 20</t>
   </si>
 </sst>
 </file>
@@ -306,9 +306,10 @@
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -330,10 +331,10 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -356,10 +357,10 @@
       <c r="F2" s="1" t="n">
         <v>123456789</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -382,10 +383,10 @@
       <c r="F3" s="1" t="n">
         <v>999888777</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>